<commit_message>
samples(lem 12): the rapid-drawdown sample is built by tools/build_johnson_rapid.py on the COMBO-2 family (core-only d/ψ 250/14, circle 275/235 R160) and stays the two-steady anchor; seven locks moved (Spencer 1.646 → 1.498)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_johnson_rapid_KEY.xlsx
+++ b/docs/lem/files/xslope_johnson_rapid_KEY.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11708D50-B4AE-4447-916E-877A7873BC20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523500CF-89B8-4644-B955-31C74218CF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="33220" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4560" yWindow="4320" windowWidth="46940" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -223,6 +223,12 @@
     <t>Water loads:</t>
   </si>
   <si>
+    <t>auto</t>
+  </si>
+  <si>
+    <t>Surface family:</t>
+  </si>
+  <si>
     <t>Unit Options:</t>
   </si>
   <si>
@@ -397,9 +403,6 @@
     <t>g</t>
   </si>
   <si>
-    <t>gsat</t>
-  </si>
-  <si>
     <t>option</t>
   </si>
   <si>
@@ -463,24 +466,9 @@
     <t>hb_d</t>
   </si>
   <si>
-    <t>s(g)</t>
-  </si>
-  <si>
-    <t>s(c)</t>
-  </si>
-  <si>
     <t>s(f)</t>
   </si>
   <si>
-    <t>s(c/p)</t>
-  </si>
-  <si>
-    <t>s(d)</t>
-  </si>
-  <si>
-    <t>s(psi)</t>
-  </si>
-  <si>
     <t>k1</t>
   </si>
   <si>
@@ -874,9 +862,6 @@
     <t>H</t>
   </si>
   <si>
-    <t>qp</t>
-  </si>
-  <si>
     <t>D</t>
   </si>
   <si>
@@ -892,9 +877,6 @@
     <t>I</t>
   </si>
   <si>
-    <t>Fixity</t>
-  </si>
-  <si>
     <t>P</t>
   </si>
   <si>
@@ -991,7 +973,24 @@
     <t>save_times</t>
   </si>
   <si>
-    <t>auto</t>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(c)</t>
+    </r>
   </si>
   <si>
     <r>
@@ -1048,26 +1047,6 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t>(c)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="0"/>
-        <rFont val="Symbol"/>
-        <charset val="2"/>
-      </rPr>
-      <t>s</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="0"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>(c/p)</t>
     </r>
   </si>
@@ -1133,26 +1112,28 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <rFont val="Symbol"/>
-        <charset val="2"/>
-      </rPr>
-      <t>q</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>p</t>
-    </r>
+    <t>yr</t>
+  </si>
+  <si>
+    <t>Adhesion</t>
+  </si>
+  <si>
+    <t>Delta</t>
+  </si>
+  <si>
+    <t>1D element size:</t>
+  </si>
+  <si>
+    <t>Head</t>
+  </si>
+  <si>
+    <t>Tip</t>
+  </si>
+  <si>
+    <t>Pinned</t>
+  </si>
+  <si>
+    <t>Unrotated</t>
   </si>
 </sst>
 </file>
@@ -1919,6 +1900,645 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>217714</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>54430</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>444500</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>90714</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B0FB8E9-E4E3-974A-BE46-8E599C58A56D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16455571" y="254001"/>
+          <a:ext cx="3855358" cy="4027713"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Label</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = name used in error messages, summaries, and plots</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>(x1, y1), (x2, y2) </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t>= start and end of reinforcement line</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Type</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = support preset, fills Dir and Appl: Geosynthetic (Tangent, Active), Nail (Axial, Passive), Tieback (Axial, Active), Anchor (Axial, Active)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Dir</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = force direction at the slip surface (LEM only): Tangent = reorients along slip surface (flexible); Axial = along the reinforcement line (rigid). Set by Type; overtype to override.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Appl</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = force application (LEM only): Active = allowable force, not divided by FS (default). Passive = ultimate force, divided by FS. Set by Type; overtype to override.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Tmax</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = tensile capacity (force/length; or force per element if Spacing is given)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Lp1, Lp2 </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t>= pullout length at end 1 / end 2 (0 = fully anchored)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Adhesion</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = soii-reinforcement interface adhesion (blank</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = use Lp)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>Delta</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = soil-reinforcement interface friction angle (blank = use Lp)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="0"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Tend1, Tend2 </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t>= anchorage/plate/connection capacity at end 1 / end 2 (0 = friction only)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Spacing</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = out-of-plane spacing for discrete supports (nails, tiebacks); blank or 1 for geosynthetics</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Tres</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = residual capacity after rupture (FEM only)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>E</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = modulus of elasticity of reinforcement (FEM only)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Area</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = cross-sectional area of reinforcement (FEM only)</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="0"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>290286</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>126999</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>553358</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>54428</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C6B716B0-439A-6440-8742-7BC140EF924C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14205857" y="126999"/>
+          <a:ext cx="3156858" cy="2521858"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>(x1,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t> y1), (x2, y2) </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>= top and bottom of pile</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>H</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> = Pile force magnitude (kN/m or lb/ft). </a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>appl</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> = force application (LEM only): Active = allowable force, not divided by FS (default). Passive = ultimate force, divided by FS.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>D</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t> = </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Pile diameter</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> (ft or m)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>S</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t> = center to center pile spacing</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> (ft or m)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Vcap</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> = Shear</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> capacity of pile (force)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Mcap</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> = Moment capacity of pile (force x length)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>E</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> = Young's modulus of pile material (force/lengh^2)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>I </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>= </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Moment of inertia (length^4)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>Area</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> = </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Cross-sectional area (length^2)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Head</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> = Pile head fixity status</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Tip</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> = Pile tip fixity status</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2236,7 +2856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.6640625" customWidth="1"/>
@@ -2261,7 +2881,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="30">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -2437,7 +3057,7 @@
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C20" s="14" t="s">
-        <v>45</v>
+        <v>313</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>46</v>
@@ -2449,7 +3069,7 @@
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C21" s="14" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>49</v>
@@ -2461,33 +3081,43 @@
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C22" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="D22" s="1"/>
+        <v>48</v>
+      </c>
       <c r="F22" s="1"/>
+      <c r="D22"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="1"/>
       <c r="C23" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" s="1"/>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B24" s="1"/>
+      <c r="C24" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B24" s="1"/>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="C25" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25"/>
     </row>
     <row r="49" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D49" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="50" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D50" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="51" spans="4:4" x14ac:dyDescent="0.2">
@@ -2497,22 +3127,22 @@
     </row>
     <row r="53" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D53" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="54" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D54" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="55" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D55" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="56" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D56" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="57" spans="4:4" x14ac:dyDescent="0.2">
@@ -2520,121 +3150,129 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D59" s="1" t="s">
-        <v>60</v>
+    <row r="58" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D58" s="1" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="60" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D60" s="1" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
     </row>
     <row r="61" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D61" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="63" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D63" s="1" t="s">
-        <v>62</v>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="62" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D62" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="64" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D64" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="65" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D65" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="66" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D66" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="67" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D67" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="68" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D68" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="69" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D69" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="70" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D70" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="71" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D71" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="73" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D73" s="1" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="72" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D72" s="1" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="74" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D74" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="75" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D75" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="76" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D76" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="77" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D77" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="78" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D78" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D79" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B7:D7"/>
   </mergeCells>
-  <dataValidations count="7">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D22" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D23" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"rollers,fixed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>$D$50:$D$51</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D9" xr:uid="{00000000-0002-0000-0000-000002000000}">
-      <formula1>$D$54:$D$57</formula1>
+      <formula1>$D$54:$D$58</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D17" xr:uid="{00000000-0002-0000-0000-000003000000}">
-      <formula1>$D$60:$D$61</formula1>
+      <formula1>$D$61:$D$62</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D14" xr:uid="{00000000-0002-0000-0000-000004000000}">
-      <formula1>$D$64:$D$71</formula1>
+      <formula1>$D$65:$D$72</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D18" xr:uid="{00000000-0002-0000-0000-000005000000}">
-      <formula1>$D$74:$D$78</formula1>
+      <formula1>$D$75:$D$79</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D23" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D24" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"auto,manual"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="D25" xr:uid="{00000000-0002-0000-0000-000007000000}">
+      <formula1>"circular,non-circular"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2643,83 +3281,89 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A2:AB25"/>
+  <dimension ref="A2:AD25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
     <col min="2" max="6" width="10.83203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="13.1640625" customWidth="1"/>
-    <col min="10" max="12" width="10.83203125" style="1" customWidth="1"/>
-    <col min="16" max="18" width="10.83203125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="4.33203125" customWidth="1"/>
+    <col min="10" max="14" width="10.83203125" style="1" customWidth="1"/>
+    <col min="18" max="20" width="10.83203125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="4.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="F2" s="12" t="s">
         <v>246</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="G2" s="40" t="s">
         <v>247</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="H2" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="I2" s="40" t="s">
         <v>249</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="J2" s="27" t="s">
         <v>250</v>
       </c>
-      <c r="G2" s="40" t="s">
+      <c r="K2" s="27" t="s">
         <v>251</v>
       </c>
-      <c r="H2" s="40" t="s">
+      <c r="L2" s="27" t="s">
         <v>252</v>
       </c>
-      <c r="I2" s="40" t="s">
+      <c r="M2" s="27" t="s">
+        <v>311</v>
+      </c>
+      <c r="N2" s="27" t="s">
+        <v>312</v>
+      </c>
+      <c r="O2" s="27" t="s">
         <v>253</v>
       </c>
-      <c r="J2" s="27" t="s">
+      <c r="P2" s="27" t="s">
         <v>254</v>
       </c>
-      <c r="K2" s="27" t="s">
+      <c r="Q2" s="27" t="s">
         <v>255</v>
       </c>
-      <c r="L2" s="27" t="s">
+      <c r="R2" s="28" t="s">
         <v>256</v>
       </c>
-      <c r="M2" s="27" t="s">
+      <c r="S2" s="28" t="s">
+        <v>122</v>
+      </c>
+      <c r="T2" s="28" t="s">
         <v>257</v>
       </c>
-      <c r="N2" s="27" t="s">
+      <c r="AB2" t="s">
         <v>258</v>
       </c>
-      <c r="O2" s="27" t="s">
+      <c r="AC2" t="s">
         <v>259</v>
       </c>
-      <c r="P2" s="28" t="s">
+      <c r="AD2" t="s">
         <v>260</v>
       </c>
-      <c r="Q2" s="28" t="s">
-        <v>121</v>
-      </c>
-      <c r="R2" s="28" t="s">
-        <v>261</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>262</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>263</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -2730,11 +3374,11 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3" t="str">
-        <f t="shared" ref="H3:H22" si="0">IF($G3="","",IFERROR(VLOOKUP($G3,$Z$8:$AB$11,2,0),""))</f>
+        <f t="shared" ref="H3:H22" si="0">IF($G3="","",IFERROR(VLOOKUP($G3,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I3" s="3" t="str">
-        <f t="shared" ref="I3:I22" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$Z$8:$AB$11,3,0),""))</f>
+        <f t="shared" ref="I3:I22" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$AB$8:$AD$11,3,0),""))</f>
         <v/>
       </c>
       <c r="J3" s="3"/>
@@ -2746,17 +3390,19 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="R3" s="3"/>
-      <c r="Z3" t="s">
-        <v>265</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>266</v>
-      </c>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
       <c r="AB3" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>262</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -2783,11 +3429,13 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
-      <c r="Z4" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="AB4" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -2814,11 +3462,13 @@
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
-      <c r="Z5" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="AB5" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -2845,8 +3495,10 @@
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S6" s="3"/>
+      <c r="T6" s="3"/>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -2873,8 +3525,10 @@
       <c r="P7" s="3"/>
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S7" s="3"/>
+      <c r="T7" s="3"/>
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -2901,17 +3555,19 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
-      <c r="Z8" t="s">
-        <v>262</v>
-      </c>
-      <c r="AA8" t="s">
-        <v>263</v>
-      </c>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
       <c r="AB8" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
+        <v>258</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>259</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -2938,17 +3594,19 @@
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
-      <c r="Z9" t="s">
-        <v>265</v>
-      </c>
-      <c r="AA9" t="s">
-        <v>266</v>
-      </c>
+      <c r="S9" s="3"/>
+      <c r="T9" s="3"/>
       <c r="AB9" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>262</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -2975,17 +3633,19 @@
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
       <c r="R10" s="3"/>
-      <c r="Z10" t="s">
-        <v>268</v>
-      </c>
-      <c r="AA10" t="s">
-        <v>266</v>
-      </c>
+      <c r="S10" s="3"/>
+      <c r="T10" s="3"/>
       <c r="AB10" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC10" t="s">
+        <v>262</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -3012,17 +3672,19 @@
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
-      <c r="Z11" t="s">
-        <v>269</v>
-      </c>
-      <c r="AA11" t="s">
-        <v>266</v>
-      </c>
+      <c r="S11" s="3"/>
+      <c r="T11" s="3"/>
       <c r="AB11" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
+        <v>265</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>262</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -3049,8 +3711,10 @@
       <c r="P12" s="3"/>
       <c r="Q12" s="3"/>
       <c r="R12" s="3"/>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S12" s="3"/>
+      <c r="T12" s="3"/>
+    </row>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -3077,8 +3741,10 @@
       <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
       <c r="R13" s="3"/>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S13" s="3"/>
+      <c r="T13" s="3"/>
+    </row>
+    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -3105,8 +3771,10 @@
       <c r="P14" s="3"/>
       <c r="Q14" s="3"/>
       <c r="R14" s="3"/>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S14" s="3"/>
+      <c r="T14" s="3"/>
+    </row>
+    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -3133,8 +3801,10 @@
       <c r="P15" s="3"/>
       <c r="Q15" s="3"/>
       <c r="R15" s="3"/>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S15" s="3"/>
+      <c r="T15" s="3"/>
+    </row>
+    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -3161,8 +3831,10 @@
       <c r="P16" s="3"/>
       <c r="Q16" s="3"/>
       <c r="R16" s="3"/>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="S16" s="3"/>
+      <c r="T16" s="3"/>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -3189,8 +3861,10 @@
       <c r="P17" s="3"/>
       <c r="Q17" s="3"/>
       <c r="R17" s="3"/>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="S17" s="3"/>
+      <c r="T17" s="3"/>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -3217,8 +3891,10 @@
       <c r="P18" s="3"/>
       <c r="Q18" s="3"/>
       <c r="R18" s="3"/>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -3245,8 +3921,10 @@
       <c r="P19" s="3"/>
       <c r="Q19" s="3"/>
       <c r="R19" s="3"/>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="S19" s="3"/>
+      <c r="T19" s="3"/>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -3273,8 +3951,10 @@
       <c r="P20" s="3"/>
       <c r="Q20" s="3"/>
       <c r="R20" s="3"/>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="S20" s="3"/>
+      <c r="T20" s="3"/>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -3301,8 +3981,10 @@
       <c r="P21" s="3"/>
       <c r="Q21" s="3"/>
       <c r="R21" s="3"/>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="S21" s="3"/>
+      <c r="T21" s="3"/>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -3329,115 +4011,118 @@
       <c r="P22" s="3"/>
       <c r="Q22" s="3"/>
       <c r="R22" s="3"/>
-    </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="T23" s="42"/>
-      <c r="U23" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="S22" s="3"/>
+      <c r="T22" s="3"/>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="V23" s="42"/>
+      <c r="W23" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
-      <c r="T24" s="26"/>
-      <c r="U24" s="9" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V24" s="26"/>
+      <c r="W24" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
       <c r="K25" s="9"/>
       <c r="L25" s="9"/>
-      <c r="T25" s="29"/>
-      <c r="U25" s="9" t="s">
-        <v>102</v>
+      <c r="V25" s="29"/>
+      <c r="W25" s="9" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G22" xr:uid="{00000000-0002-0000-0900-000000000000}">
-      <formula1>$Z$2:$Z$5</formula1>
+      <formula1>$AB$2:$AB$5</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H22" xr:uid="{00000000-0002-0000-0900-000001000000}">
-      <formula1>$AA$2:$AA$3</formula1>
+      <formula1>$AC$2:$AC$3</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I22" xr:uid="{00000000-0002-0000-0900-000002000000}">
-      <formula1>$AB$2:$AB$3</formula1>
+      <formula1>$AD$2:$AD$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A2:AA18"/>
+  <dimension ref="A2:AA17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.5" style="1" customWidth="1"/>
-    <col min="3" max="8" width="10.83203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5" customWidth="1"/>
-    <col min="10" max="17" width="10.83203125" style="1" customWidth="1"/>
+    <col min="3" max="7" width="10.83203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5" customWidth="1"/>
+    <col min="9" max="17" width="10.83203125" style="1" customWidth="1"/>
     <col min="18" max="18" width="5.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="F2" s="12" t="s">
         <v>246</v>
       </c>
-      <c r="C2" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="E2" s="12" t="s">
+      <c r="G2" s="40" t="s">
+        <v>266</v>
+      </c>
+      <c r="H2" s="40" t="s">
         <v>249</v>
       </c>
-      <c r="F2" s="12" t="s">
-        <v>250</v>
-      </c>
-      <c r="G2" s="40" t="s">
+      <c r="I2" s="27" t="s">
+        <v>267</v>
+      </c>
+      <c r="J2" s="27" t="s">
+        <v>268</v>
+      </c>
+      <c r="K2" s="41" t="s">
+        <v>269</v>
+      </c>
+      <c r="L2" s="41" t="s">
         <v>270</v>
       </c>
-      <c r="H2" s="40" t="s">
-        <v>317</v>
-      </c>
-      <c r="I2" s="40" t="s">
-        <v>253</v>
-      </c>
-      <c r="J2" s="27" t="s">
-        <v>272</v>
-      </c>
-      <c r="K2" s="27" t="s">
-        <v>273</v>
-      </c>
-      <c r="L2" s="41" t="s">
-        <v>274</v>
-      </c>
-      <c r="M2" s="41" t="s">
-        <v>275</v>
+      <c r="M2" s="28" t="s">
+        <v>122</v>
       </c>
       <c r="N2" s="28" t="s">
-        <v>121</v>
+        <v>271</v>
       </c>
       <c r="O2" s="28" t="s">
-        <v>276</v>
+        <v>257</v>
       </c>
       <c r="P2" s="28" t="s">
-        <v>261</v>
+        <v>314</v>
       </c>
       <c r="Q2" s="28" t="s">
-        <v>277</v>
+        <v>315</v>
       </c>
       <c r="Z2" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="AA2" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.2">
@@ -3461,10 +4146,10 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="Z3" t="s">
-        <v>230</v>
+        <v>316</v>
       </c>
       <c r="AA3" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.2">
@@ -3487,6 +4172,9 @@
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
+      <c r="Z4" t="s">
+        <v>317</v>
+      </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
@@ -3508,6 +4196,9 @@
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
+      <c r="Z5" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
@@ -3657,41 +4348,38 @@
       <c r="Q12" s="3"/>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="I14" s="9"/>
       <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
+      <c r="S15" s="42"/>
+      <c r="T15" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="S16" s="42"/>
-      <c r="T16" t="s">
-        <v>89</v>
+      <c r="S16" s="26"/>
+      <c r="T16" s="9" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="19:20" x14ac:dyDescent="0.2">
-      <c r="S17" s="26"/>
+      <c r="S17" s="29"/>
       <c r="T17" s="9" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="18" spans="19:20" x14ac:dyDescent="0.2">
-      <c r="S18" s="29"/>
-      <c r="T18" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q3:Q12" xr:uid="{00000000-0002-0000-0A00-000000000000}">
-      <formula1>$Z$2:$Z$3</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H12" xr:uid="{00000000-0002-0000-0A00-000001000000}">
+      <formula1>$AA$2:$AA$3</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I12" xr:uid="{00000000-0002-0000-0A00-000001000000}">
-      <formula1>$AA$2:$AA$3</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P3:Q12" xr:uid="{00000000-0002-0000-0A00-000000000000}">
+      <formula1>$Z$2:$Z$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3707,22 +4395,22 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -3945,27 +4633,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="64" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="59" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="59" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="59" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="59" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="59" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -3989,63 +4677,63 @@
         <v>100.0</v>
       </c>
       <c r="K3" s="32" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="L3" s="33"/>
       <c r="N3" s="32" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="O3" s="33"/>
       <c r="Q3" s="32" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="R3" s="33"/>
       <c r="T3" s="6" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="H4" s="25" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="I4" s="25" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="K4" s="25" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="L4" s="25" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="N4" s="25" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="O4" s="25" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="Q4" s="25" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="R4" s="25" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="U4" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -4074,10 +4762,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="U5" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -4106,7 +4794,7 @@
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
       <c r="T6" s="1" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="U6" s="9"/>
     </row>
@@ -4399,27 +5087,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="68" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="60" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="60" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="60" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="60" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="60" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -4443,63 +5131,63 @@
         <v>100.0</v>
       </c>
       <c r="K3" s="34" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="L3" s="35"/>
       <c r="N3" s="34" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="O3" s="35"/>
       <c r="Q3" s="34" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="R3" s="35"/>
       <c r="T3" s="6" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="H4" s="25" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="I4" s="25" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="K4" s="25" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="L4" s="25" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="N4" s="25" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="O4" s="25" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="Q4" s="25" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="R4" s="25" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="U4" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -4528,10 +5216,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="U5" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -4846,22 +5534,22 @@
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B2" s="50" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="C2" s="50" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="D2" s="50" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="E2" s="50" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="F2" s="50" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="G2" s="50" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.2">
@@ -4872,7 +5560,7 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="I3" s="14" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="J3" s="3"/>
     </row>
@@ -4894,7 +5582,7 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="I5" s="14" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="J5" s="3"/>
     </row>
@@ -4916,7 +5604,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="I7" s="14" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -4928,7 +5616,7 @@
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="I8" s="14" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="J8" s="3"/>
     </row>
@@ -4940,7 +5628,7 @@
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="I9" s="14" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="J9" s="3"/>
     </row>
@@ -4960,7 +5648,7 @@
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="J11" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
@@ -5782,123 +6470,123 @@
   <sheetData>
     <row r="2" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C2" s="6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="AD2" s="6"/>
       <c r="AJ2" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="P3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="AD3" s="14"/>
       <c r="AJ3" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AK3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C4" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="L4" s="42"/>
       <c r="M4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="O4" s="1" t="s">
         <v>18</v>
       </c>
       <c r="P4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AD4" s="14"/>
       <c r="AJ4" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="AK4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C5" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="L5" s="26"/>
       <c r="M5" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="P5" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AD5" s="14"/>
       <c r="AJ5" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AK5" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C6" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="L6" s="29"/>
       <c r="M6" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="P6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="AE6" s="1"/>
       <c r="AF6" s="1"/>
     </row>
     <row r="7" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C7" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="AE7" s="1"/>
       <c r="AF7" s="1"/>
     </row>
     <row r="9" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C9" s="53" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D9" s="52"/>
       <c r="E9" s="52"/>
@@ -5924,7 +6612,7 @@
       <c r="Y9" s="54"/>
       <c r="Z9" s="54"/>
       <c r="AA9" s="53" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="AB9" s="54"/>
       <c r="AC9" s="54"/>
@@ -5932,7 +6620,7 @@
       <c r="AE9" s="54"/>
       <c r="AF9" s="54"/>
       <c r="AG9" s="53" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="AH9" s="54"/>
       <c r="AI9" s="54"/>
@@ -5949,127 +6637,127 @@
         <v>8</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C10" s="45" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D10" s="48" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="E10" s="44" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F10" s="44" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G10" s="45" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H10" s="44" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I10" s="44" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J10" s="49" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K10" s="49" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="L10" s="21" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="M10" s="21" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N10" s="43" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O10" s="44" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P10" s="44" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="Q10" s="44" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="R10" s="44" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="S10" s="44" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="T10" s="44" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="U10" s="44" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="V10" s="44" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="W10" s="44" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="X10" s="44" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Y10" s="44" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="Z10" s="44" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="AA10" s="46" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="AB10" s="46" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="AC10" s="47" t="s">
+        <v>135</v>
+      </c>
+      <c r="AD10" s="46" t="s">
+        <v>306</v>
+      </c>
+      <c r="AE10" s="46" t="s">
+        <v>307</v>
+      </c>
+      <c r="AF10" s="47" t="s">
+        <v>308</v>
+      </c>
+      <c r="AG10" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="AD10" s="46" t="s">
-        <v>313</v>
-      </c>
-      <c r="AE10" s="46" t="s">
-        <v>314</v>
-      </c>
-      <c r="AF10" s="47" t="s">
-        <v>315</v>
-      </c>
-      <c r="AG10" s="23" t="s">
+      <c r="AH10" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="AI10" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="AJ10" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="AK10" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="AH10" s="23" t="s">
+      <c r="AL10" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="AI10" s="23" t="s">
+      <c r="AM10" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="AJ10" s="23" t="s">
+      <c r="AN10" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="AK10" s="23" t="s">
+      <c r="AO10" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="AL10" s="23" t="s">
+      <c r="AP10" s="23" t="s">
         <v>145</v>
-      </c>
-      <c r="AM10" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="AN10" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="AO10" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="AP10" s="23" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="11" spans="1:42" x14ac:dyDescent="0.2">
@@ -6227,10 +6915,10 @@
         <v>0.0</v>
       </c>
       <c r="J12" s="3">
-        <v>500.0</v>
+        <v>250.0</v>
       </c>
       <c r="K12" s="3">
-        <v>12.0</v>
+        <v>14.0</v>
       </c>
       <c r="L12" s="3"/>
       <c r="M12" s="3">
@@ -6351,10 +7039,10 @@
         <v>0.0</v>
       </c>
       <c r="J13" s="3">
-        <v>250.0</v>
+        <v>0.0</v>
       </c>
       <c r="K13" s="3">
-        <v>20.0</v>
+        <v>0.0</v>
       </c>
       <c r="L13" s="3"/>
       <c r="M13" s="3">
@@ -7784,16 +8472,16 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B2" s="3">
         <v>0.0</v>
       </c>
       <c r="D2" s="24" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="N2" s="24" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
@@ -7816,157 +8504,157 @@
       </c>
       <c r="H4" s="52"/>
       <c r="J4" s="55" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="K4" s="52"/>
       <c r="M4" s="55" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="N4" s="52"/>
       <c r="P4" s="55" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
       <c r="S4" s="55" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="T4" s="54"/>
       <c r="U4" s="1"/>
       <c r="V4" s="55" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="W4" s="54"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="55" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="55" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="AC4" s="54"/>
       <c r="AE4" s="55" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="55" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
       <c r="AK4" s="55" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="55" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
       <c r="AQ4" s="55" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B5" s="37">
         <v>1</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E5" s="37">
         <v>2</v>
       </c>
       <c r="G5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="H5" s="37">
         <v>3</v>
       </c>
       <c r="J5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="K5" s="37">
         <v>4</v>
       </c>
       <c r="M5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="N5" s="37">
         <v>5</v>
       </c>
       <c r="P5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="Q5" s="37">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="T5" s="37">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="W5" s="37">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="Z5" s="37">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="AC5" s="37">
         <v>10</v>
       </c>
       <c r="AE5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="AF5" s="37">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="AI5" s="37">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="AL5" s="37">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="AO5" s="37">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="AR5" s="37">
         <v>15</v>
@@ -8059,172 +8747,172 @@
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B7" s="37"/>
       <c r="D7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E7" s="37"/>
       <c r="G7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="H7" s="37"/>
       <c r="J7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="K7" s="37"/>
       <c r="M7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="N7" s="37"/>
       <c r="P7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="Q7" s="37"/>
       <c r="R7" s="1"/>
       <c r="S7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="T7" s="37"/>
       <c r="U7" s="1"/>
       <c r="V7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="W7" s="37"/>
       <c r="X7" s="1"/>
       <c r="Y7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="Z7" s="37"/>
       <c r="AA7" s="1"/>
       <c r="AB7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="AC7" s="37"/>
       <c r="AE7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="AF7" s="37"/>
       <c r="AG7" s="1"/>
       <c r="AH7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="AI7" s="37"/>
       <c r="AJ7" s="1"/>
       <c r="AK7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="AL7" s="37"/>
       <c r="AM7" s="1"/>
       <c r="AN7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="AO7" s="37"/>
       <c r="AP7" s="1"/>
       <c r="AQ7" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="AR7" s="37"/>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="R8" s="1"/>
       <c r="S8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="U8" s="1"/>
       <c r="V8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="W8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="X8" s="1"/>
       <c r="Y8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="Z8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AA8" s="1"/>
       <c r="AB8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AC8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AE8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AF8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AG8" s="1"/>
       <c r="AH8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AI8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AJ8" s="1"/>
       <c r="AK8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AL8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AM8" s="1"/>
       <c r="AN8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AO8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AP8" s="1"/>
       <c r="AQ8" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AR8" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
@@ -9098,27 +9786,27 @@
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="P6:Q6"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="P4:Q4"/>
     <mergeCell ref="Y4:Z4"/>
     <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="A6:B6"/>
     <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="P6:Q6"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9152,277 +9840,277 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A4" s="55" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B4" s="52"/>
       <c r="D4" s="55" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="E4" s="52"/>
       <c r="G4" s="55" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="H4" s="52"/>
       <c r="J4" s="55" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="K4" s="52"/>
       <c r="M4" s="55" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="N4" s="52"/>
       <c r="P4" s="55" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
       <c r="S4" s="55" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="T4" s="54"/>
       <c r="U4" s="1"/>
       <c r="V4" s="55" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="W4" s="54"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="55" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="55" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="AC4" s="54"/>
       <c r="AE4" s="55" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="55" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
       <c r="AK4" s="55" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="55" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
       <c r="AQ4" s="55" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="E5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="G5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="H5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="J5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="M5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="N5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="P5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="Q5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="T5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="W5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="Z5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="AC5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="AE5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="AF5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="AI5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="AL5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="AO5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="AR5" s="39" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B6" s="39">
         <v>1</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E6" s="39">
         <v>2</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="H6" s="39">
         <v>3</v>
       </c>
       <c r="J6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="K6" s="39">
         <v>4</v>
       </c>
       <c r="M6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="N6" s="39">
         <v>5</v>
       </c>
       <c r="P6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="Q6" s="39">
         <v>6</v>
       </c>
       <c r="R6" s="1"/>
       <c r="S6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="T6" s="39">
         <v>7</v>
       </c>
       <c r="U6" s="1"/>
       <c r="V6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="W6" s="39">
         <v>8</v>
       </c>
       <c r="X6" s="1"/>
       <c r="Y6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="Z6" s="39">
         <v>9</v>
       </c>
       <c r="AA6" s="1"/>
       <c r="AB6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="AC6" s="39">
         <v>10</v>
       </c>
       <c r="AE6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="AF6" s="39">
         <v>11</v>
       </c>
       <c r="AG6" s="1"/>
       <c r="AH6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="AI6" s="39">
         <v>12</v>
       </c>
       <c r="AJ6" s="1"/>
       <c r="AK6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="AL6" s="39">
         <v>13</v>
       </c>
       <c r="AM6" s="1"/>
       <c r="AN6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="AO6" s="39">
         <v>14</v>
       </c>
       <c r="AP6" s="1"/>
       <c r="AQ6" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="AR6" s="39">
         <v>15</v>
@@ -9515,172 +10203,172 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B8" s="39"/>
       <c r="D8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E8" s="39"/>
       <c r="G8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="H8" s="39"/>
       <c r="J8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="K8" s="39"/>
       <c r="M8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="N8" s="39"/>
       <c r="P8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="Q8" s="39"/>
       <c r="R8" s="1"/>
       <c r="S8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="T8" s="39"/>
       <c r="U8" s="1"/>
       <c r="V8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="W8" s="39"/>
       <c r="X8" s="1"/>
       <c r="Y8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="Z8" s="39"/>
       <c r="AA8" s="1"/>
       <c r="AB8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="AC8" s="39"/>
       <c r="AE8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="AF8" s="39"/>
       <c r="AG8" s="1"/>
       <c r="AH8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="AI8" s="39"/>
       <c r="AJ8" s="1"/>
       <c r="AK8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="AL8" s="39"/>
       <c r="AM8" s="1"/>
       <c r="AN8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="AO8" s="39"/>
       <c r="AP8" s="1"/>
       <c r="AQ8" s="38" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="AR8" s="39"/>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="R9" s="1"/>
       <c r="S9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="U9" s="1"/>
       <c r="V9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="W9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="X9" s="1"/>
       <c r="Y9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="Z9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AA9" s="1"/>
       <c r="AB9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AC9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AE9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AF9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AG9" s="1"/>
       <c r="AH9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AI9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AJ9" s="1"/>
       <c r="AK9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AL9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AM9" s="1"/>
       <c r="AN9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AO9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AP9" s="1"/>
       <c r="AQ9" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AR9" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
@@ -10485,36 +11173,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AN7:AO7"/>
-    <mergeCell ref="M4:N4"/>
     <mergeCell ref="S4:T4"/>
-    <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="J4:K4"/>
     <mergeCell ref="Y7:Z7"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="D4:E4"/>
     <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="P4:Q4"/>
     <mergeCell ref="Y4:Z4"/>
     <mergeCell ref="AE7:AF7"/>
     <mergeCell ref="AK7:AL7"/>
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN7:AO7"/>
+    <mergeCell ref="AH7:AI7"/>
+    <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="V7:W7"/>
+    <mergeCell ref="P7:Q7"/>
     <mergeCell ref="AB7:AC7"/>
-    <mergeCell ref="AH7:AI7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
     <cfRule type="expression" dxfId="17" priority="1">
@@ -10611,20 +11299,20 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="59" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B2" s="54"/>
       <c r="D2" s="60" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="E2" s="54"/>
       <c r="G2" s="22" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="32" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B3" s="33" t="inlineStr">
         <is>
@@ -10632,7 +11320,7 @@
         </is>
       </c>
       <c r="D3" s="34" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="E3" s="35" t="inlineStr">
         <is>
@@ -10643,19 +11331,19 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="H4" s="1"/>
     </row>
@@ -10668,7 +11356,7 @@
         <v>18</v>
       </c>
       <c r="H5" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -10677,10 +11365,10 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="G6" s="1" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="H6" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -10817,31 +11505,31 @@
   <sheetData>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="E2" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="F2" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="G2" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="H2" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="J2" s="5" t="s">
         <v>202</v>
-      </c>
-      <c r="F2" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="G2" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="H2" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>206</v>
       </c>
       <c r="K2" s="10" t="s">
         <v>5</v>
@@ -10852,10 +11540,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>280.0</v>
+        <v>275.0</v>
       </c>
       <c r="C3" s="3">
-        <v>270.0</v>
+        <v>235.0</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
@@ -10863,16 +11551,16 @@
         </is>
       </c>
       <c r="E3" s="3">
-        <v>50.0</v>
+        <v>75.0</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="J3" s="1" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
@@ -10887,10 +11575,10 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="J4" s="1" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -10905,10 +11593,10 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="J5" s="1" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="K5" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -10935,7 +11623,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="J7" s="5" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -10950,7 +11638,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="J8" s="14" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="K8"/>
     </row>
@@ -10966,7 +11654,7 @@
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="J9" s="14" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="K9"/>
     </row>
@@ -10982,7 +11670,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="J10" s="14" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="K10"/>
     </row>
@@ -10998,7 +11686,7 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="J11" s="14" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="K11"/>
     </row>
@@ -11014,31 +11702,31 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="J12" s="14" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="K12"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J13" s="14" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="K13"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J14" s="14" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="K14"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J15" s="14" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="K15"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J16" s="14" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
@@ -11047,7 +11735,7 @@
     </row>
     <row r="17" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J17" s="14" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="K17"/>
     </row>
@@ -11088,16 +11776,16 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>5</v>
@@ -11108,10 +11796,10 @@
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="F3" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -11119,10 +11807,10 @@
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="E4" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="F4" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -11130,10 +11818,10 @@
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="E5" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="F5" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -11257,128 +11945,128 @@
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B2" t="str">
-        <f>IF(main!$D$23="auto","Enter non-water loads only — water loads derive automatically from the piezometric line / seepage boundary conditions.","")</f>
+        <f>IF(main!$D$24="auto","Enter non-water loads only — water loads derive automatically from the piezometric line / seepage boundary conditions.","")</f>
         <v>Enter non-water loads only — water loads derive automatically from the piezometric line / seepage boundary conditions.</v>
       </c>
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B4" s="61" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="C4" s="62"/>
       <c r="D4" s="62"/>
       <c r="F4" s="61" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="G4" s="62"/>
       <c r="H4" s="62"/>
       <c r="J4" s="61" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="K4" s="62"/>
       <c r="L4" s="62"/>
       <c r="N4" s="61" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="O4" s="62"/>
       <c r="P4" s="62"/>
       <c r="R4" s="61" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="S4" s="62"/>
       <c r="T4" s="62"/>
       <c r="V4" s="61" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="W4" s="62"/>
       <c r="X4" s="62"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="58" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C5" s="57"/>
       <c r="D5" s="39"/>
       <c r="F5" s="58" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="G5" s="57"/>
       <c r="H5" s="39"/>
       <c r="J5" s="58" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="K5" s="57"/>
       <c r="L5" s="39"/>
       <c r="N5" s="58" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="O5" s="57"/>
       <c r="P5" s="39"/>
       <c r="R5" s="58" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="S5" s="57"/>
       <c r="T5" s="39"/>
       <c r="V5" s="58" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="W5" s="57"/>
       <c r="X5" s="39"/>
     </row>
     <row r="6" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="W6" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="X6" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.2">
@@ -11763,18 +12451,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="B4:D4"/>
     <mergeCell ref="V5:W5"/>
+    <mergeCell ref="F4:H4"/>
     <mergeCell ref="V4:X4"/>
-    <mergeCell ref="R4:T4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:O5"/>
     <mergeCell ref="R5:S5"/>
-    <mergeCell ref="F5:G5"/>
     <mergeCell ref="J5:K5"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="N5:O5"/>
-    <mergeCell ref="N4:P4"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5 H5 L5 P5 T5 X5" xr:uid="{00000000-0002-0000-0700-000000000000}">
@@ -11806,128 +12494,128 @@
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B2" t="str">
-        <f>IF(main!$D$23="auto","Enter non-water loads only — water loads derive automatically from the piezometric line / seepage boundary conditions.","")</f>
+        <f>IF(main!$D$24="auto","Enter non-water loads only — water loads derive automatically from the piezometric line / seepage boundary conditions.","")</f>
         <v>Enter non-water loads only — water loads derive automatically from the piezometric line / seepage boundary conditions.</v>
       </c>
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B4" s="63" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="C4" s="62"/>
       <c r="D4" s="62"/>
       <c r="F4" s="63" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="G4" s="62"/>
       <c r="H4" s="62"/>
       <c r="J4" s="63" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="K4" s="62"/>
       <c r="L4" s="62"/>
       <c r="N4" s="63" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="O4" s="62"/>
       <c r="P4" s="62"/>
       <c r="R4" s="63" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="S4" s="62"/>
       <c r="T4" s="62"/>
       <c r="V4" s="63" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="W4" s="62"/>
       <c r="X4" s="62"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="58" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C5" s="57"/>
       <c r="D5" s="39"/>
       <c r="F5" s="58" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="G5" s="57"/>
       <c r="H5" s="39"/>
       <c r="J5" s="58" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="K5" s="57"/>
       <c r="L5" s="39"/>
       <c r="N5" s="58" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="O5" s="57"/>
       <c r="P5" s="39"/>
       <c r="R5" s="58" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="S5" s="57"/>
       <c r="T5" s="39"/>
       <c r="V5" s="58" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="W5" s="57"/>
       <c r="X5" s="39"/>
     </row>
     <row r="6" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="W6" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="X6" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.2">
@@ -12312,18 +13000,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="B4:D4"/>
     <mergeCell ref="V5:W5"/>
+    <mergeCell ref="F4:H4"/>
     <mergeCell ref="V4:X4"/>
-    <mergeCell ref="R4:T4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:O5"/>
     <mergeCell ref="R5:S5"/>
-    <mergeCell ref="F5:G5"/>
     <mergeCell ref="J5:K5"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="N5:O5"/>
-    <mergeCell ref="N4:P4"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5 H5 L5 P5 T5 X5" xr:uid="{00000000-0002-0000-0800-000000000000}">

</xml_diff>